<commit_message>
Improved precondition parsing and Selector map
</commit_message>
<xml_diff>
--- a/outputs/qa_testing_agent/test_inputs/devops_tests.xlsx
+++ b/outputs/qa_testing_agent/test_inputs/devops_tests.xlsx
@@ -526,17 +526,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Happy Path Export Assets</t>
+          <t>HAPPY_PATH - Auto-populate additional tags after results load</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>happy_path_export_assets</t>
+          <t>auto_populate_tags_after_results_load</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-1', 'story_title': 'Home Page: Export Assets function'}</t>
+          <t>{'story_id': 'CSV-60210', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
@@ -544,12 +544,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Navigate to the home page and perform a search to display assets.</t>
+          <t>User selects Tag A from the filter panel.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Search results are displayed with assets.</t>
+          <t>Assets associated with Tag A are displayed.</t>
         </is>
       </c>
       <c r="G2" s="2" t="n"/>
@@ -563,7 +563,7 @@
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Generated from Azure DevOps story: Home Page: Export Assets function</t>
+          <t>Ensures basic functionality of auto-populating additional tags.</t>
         </is>
       </c>
     </row>
@@ -576,12 +576,12 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Select multiple assets from the search results.</t>
+          <t>Wait for the results to finish loading.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Selected assets are highlighted or marked.</t>
+          <t>Additional tags associated with the returned assets appear in the filter panel.</t>
         </is>
       </c>
       <c r="G3" s="3" t="n"/>
@@ -596,20 +596,32 @@
       <c r="L3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>MULTI_COMBINATION - Select multiple tags for filtering</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>select_multiple_tags_for_filtering</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-60210', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+        </is>
+      </c>
       <c r="D4" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Click the 'Export' button.</t>
+          <t>User selects Tag A and Tag B from the filter panel.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>A file download of the exported assets in Excel format is initiated.</t>
+          <t>Assets associated with both Tag A and Tag B are displayed.</t>
         </is>
       </c>
       <c r="G4" s="2" t="n"/>
@@ -621,23 +633,27 @@
       <c r="I4" s="2" t="n"/>
       <c r="J4" s="2" t="n"/>
       <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="n"/>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Tests the system's ability to handle multiple tag selections.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n"/>
       <c r="B5" s="3" t="n"/>
       <c r="C5" s="3" t="n"/>
       <c r="D5" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Open the downloaded Excel file.</t>
+          <t>Wait for the results to finish loading.</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>The Excel file contains a list of the selected assets with their metadata.</t>
+          <t>Additional tags associated with the returned assets appear in the filter panel.</t>
         </is>
       </c>
       <c r="G5" s="3" t="n"/>
@@ -654,17 +670,17 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Edge Case: Export with No Assets Selected</t>
+          <t>SEQUENTIAL_REFINEMENT - Further refine results with additional tags</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>edge_case_no_assets_selected</t>
+          <t>further_refine_with_additional_tags</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-1', 'story_title': 'Home Page: Export Assets function'}</t>
+          <t>{'story_id': 'CSV-60210', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
@@ -672,12 +688,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Navigate to the home page and perform a search to display assets.</t>
+          <t>User selects Tag A from the filter panel.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Search results are displayed with assets.</t>
+          <t>Assets associated with Tag A are displayed.</t>
         </is>
       </c>
       <c r="G6" s="2" t="n"/>
@@ -691,7 +707,7 @@
       <c r="K6" s="2" t="n"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Generated from Azure DevOps story: Home Page: Export Assets function</t>
+          <t>Verifies that users can refine results using newly populated tags.</t>
         </is>
       </c>
     </row>
@@ -704,12 +720,12 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Without selecting any assets, click the 'Export' button.</t>
+          <t>Wait for the results to finish loading.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>A message is displayed informing the user to select assets before exporting.</t>
+          <t>Additional tags associated with the returned assets appear in the filter panel.</t>
         </is>
       </c>
       <c r="G7" s="3" t="n"/>
@@ -724,32 +740,20 @@
       <c r="L7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Error Scenario: Export Function Fails</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>error_scenario_export_fails</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-1', 'story_title': 'Home Page: Export Assets function'}</t>
-        </is>
-      </c>
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="n"/>
       <c r="D8" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Navigate to the home page and perform a search to display assets.</t>
+          <t>User selects an additional tag from the newly populated tags.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Search results are displayed with assets.</t>
+          <t>Assets are further filtered based on the additional tag.</t>
         </is>
       </c>
       <c r="G8" s="2" t="n"/>
@@ -761,27 +765,35 @@
       <c r="I8" s="2" t="n"/>
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>Generated from Azure DevOps story: Home Page: Export Assets function</t>
-        </is>
-      </c>
+      <c r="L8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>STATE_PERSISTENCE - User-selected tags remain highlighted</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>user_selected_tags_remain_highlighted</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-60210', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+        </is>
+      </c>
       <c r="D9" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Select multiple assets from the search results.</t>
+          <t>User selects Tag A from the filter panel.</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Selected assets are highlighted or marked.</t>
+          <t>Tag A is highlighted in the filter panel.</t>
         </is>
       </c>
       <c r="G9" s="3" t="n"/>
@@ -793,23 +805,27 @@
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
       <c r="K9" s="3" t="n"/>
-      <c r="L9" s="3" t="n"/>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>Ensures user selections persist after results load.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
       <c r="B10" s="2" t="n"/>
       <c r="C10" s="2" t="n"/>
       <c r="D10" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Click the 'Export' button.</t>
+          <t>Wait for the results to finish loading.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>An error message is displayed indicating the export could not be completed due to a server error.</t>
+          <t>Tag A remains highlighted, and additional tags appear.</t>
         </is>
       </c>
       <c r="G10" s="2" t="n"/>
@@ -826,17 +842,17 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Happy Path - Finding and Linking Duplicate Assets</t>
+          <t>BUSINESS_RULES - Display all tags associated with returned results</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>happy_path_duplicate_assets</t>
+          <t>display_all_tags_associated_with_results</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-2', 'story_title': 'Find duplicate assets'}</t>
+          <t>{'story_id': 'CSV-60210', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
@@ -844,12 +860,12 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Log in with a user account that has permissions to access the Analytics tab and asset management.</t>
+          <t>User selects Tag A from the filter panel.</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Login is successful, and the Analytics tab is accessible.</t>
+          <t>Assets associated with Tag A are displayed.</t>
         </is>
       </c>
       <c r="G11" s="3" t="n"/>
@@ -863,7 +879,7 @@
       <c r="K11" s="3" t="n"/>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>Generated from Azure DevOps story: Find duplicate assets</t>
+          <t>Validates that no tags are omitted from the filter panel.</t>
         </is>
       </c>
     </row>
@@ -876,12 +892,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Navigate to the Analytics tab.</t>
+          <t>Wait for the results to finish loading.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Analytics tab content is displayed, including the widget for duplicate assets.</t>
+          <t>All tags associated with the returned assets are displayed in the filter panel.</t>
         </is>
       </c>
       <c r="G12" s="2" t="n"/>
@@ -896,20 +912,32 @@
       <c r="L12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n"/>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>UI_UX_CONSISTENCY - Consistent styling of newly added tags</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>consistent_styling_of_newly_added_tags</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-60210', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+        </is>
+      </c>
       <c r="D13" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Trigger the vectorisation query process to find duplicate assets.</t>
+          <t>User selects Tag A from the filter panel.</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>The system processes the query and finds duplicate assets.</t>
+          <t>Assets associated with Tag A are displayed.</t>
         </is>
       </c>
       <c r="G13" s="3" t="n"/>
@@ -921,23 +949,27 @@
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
       <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="n"/>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>Checks for visual consistency in the filter panel.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
       <c r="B14" s="2" t="n"/>
       <c r="C14" s="2" t="n"/>
       <c r="D14" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Review the list of detected duplicate assets and confirm linking them together.</t>
+          <t>Wait for the results to finish loading.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>The system links duplicate assets together as specified.</t>
+          <t>Newly added tags appear with the same style as existing tags.</t>
         </is>
       </c>
       <c r="G14" s="2" t="n"/>
@@ -952,20 +984,32 @@
       <c r="L14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n"/>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>BOUNDARY_EMPTY - Handle zero results gracefully</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>handle_zero_results_gracefully</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-60210', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+        </is>
+      </c>
       <c r="D15" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Check the widget on the Analytics tab for a report on the linked duplicate assets.</t>
+          <t>User selects a tag with no associated assets.</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>The widget displays a report on the duplicate assets that were linked.</t>
+          <t>No assets are displayed, and the filter panel shows no additional tags.</t>
         </is>
       </c>
       <c r="G15" s="3" t="n"/>
@@ -977,22 +1021,26 @@
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
       <c r="K15" s="3" t="n"/>
-      <c r="L15" s="3" t="n"/>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>Tests system behavior when no results are returned.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Edge Case - No Duplicate Assets Found</t>
+          <t>ASYNC_TIMING - Seamless UI update after loading</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>edge_case_no_duplicates</t>
+          <t>seamless_ui_update_after_loading</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-2', 'story_title': 'Find duplicate assets'}</t>
+          <t>{'story_id': 'CSV-60210', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
@@ -1000,12 +1048,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Log in and navigate to the Analytics tab.</t>
+          <t>User selects Tag A from the filter panel.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Analytics tab is displayed.</t>
+          <t>Assets associated with Tag A are displayed.</t>
         </is>
       </c>
       <c r="G16" s="2" t="n"/>
@@ -1019,7 +1067,7 @@
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Generated from Azure DevOps story: Find duplicate assets</t>
+          <t>Ensures smooth UI transitions during asynchronous operations.</t>
         </is>
       </c>
     </row>
@@ -1032,12 +1080,12 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Trigger the vectorisation query process with a dataset known to have no duplicates.</t>
+          <t>Observe the UI during and after the loading process.</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>The process completes successfully.</t>
+          <t>The UI updates seamlessly without flickering or delay.</t>
         </is>
       </c>
       <c r="G17" s="3" t="n"/>
@@ -1052,20 +1100,32 @@
       <c r="L17" s="3" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n"/>
-      <c r="B18" s="2" t="n"/>
-      <c r="C18" s="2" t="n"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>ERROR_FAILURE - Network error during tag population</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>network_error_during_tag_population</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-60210', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+        </is>
+      </c>
       <c r="D18" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Check for any notifications or messages regarding the outcome of the query.</t>
+          <t>Simulate a network error after selecting Tag A.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>A message is displayed informing the user that no duplicate assets were found.</t>
+          <t>An error message is displayed, and the filter panel does not update with additional tags.</t>
         </is>
       </c>
       <c r="G18" s="2" t="n"/>
@@ -1077,22 +1137,26 @@
       <c r="I18" s="2" t="n"/>
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
-      <c r="L18" s="2" t="n"/>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Tests system resilience to network failures during tag population.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Error Scenario - System Fails to Process Query</t>
+          <t>HAPPY_PATH - Full Filter Reload on OR Operator Selection</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>error_scenario_query_failure</t>
+          <t>full_filter_reload_on_or_operator_selection</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-2', 'story_title': 'Find duplicate assets'}</t>
+          <t>{'story_id': 'CSV-27710', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -1100,12 +1164,12 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Log in and navigate to the Analytics tab.</t>
+          <t>Navigate to the Advanced Filter section and apply an initial filter.</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Analytics tab is displayed.</t>
+          <t>Initial filter is applied and visible in the filter panel.</t>
         </is>
       </c>
       <c r="G19" s="3" t="n"/>
@@ -1119,7 +1183,7 @@
       <c r="K19" s="3" t="n"/>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>Generated from Azure DevOps story: Find duplicate assets</t>
+          <t>Ensures the core functionality of filter panel reloading is working as expected.</t>
         </is>
       </c>
     </row>
@@ -1132,12 +1196,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Attempt to trigger the vectorisation query process with a valid dataset.</t>
+          <t>Select the OR operator to add an additional filter condition.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>The system attempts to process the query.</t>
+          <t>The entire filter panel reloads automatically.</t>
         </is>
       </c>
       <c r="G20" s="2" t="n"/>
@@ -1152,20 +1216,32 @@
       <c r="L20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n"/>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="3" t="n"/>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>BUSINESS_RULES - Updated Filter Options Based on Previous Selections</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>updated_filter_options_based_on_previous_selections</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-27710', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+        </is>
+      </c>
       <c r="D21" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Observe the system's behavior and response to the failed query process.</t>
+          <t>Apply a filter and then select the OR operator to add another filter.</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>The system displays an error message indicating that the query process failed and suggests possible actions or checks.</t>
+          <t>Filter panel displays updated and relevant filter options based on previously applied filters.</t>
         </is>
       </c>
       <c r="G21" s="3" t="n"/>
@@ -1177,22 +1253,26 @@
       <c r="I21" s="3" t="n"/>
       <c r="J21" s="3" t="n"/>
       <c r="K21" s="3" t="n"/>
-      <c r="L21" s="3" t="n"/>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>Verifies that new filter options are relevant to the current context.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Happy Path Password Reset</t>
+          <t>STATE_PERSISTENCE - No Loss of Existing Filters After Reload</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>happy_path_password_reset</t>
+          <t>no_loss_of_existing_filters_after_reload</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-3', 'story_title': 'User Management: Ability for user to reset password'}</t>
+          <t>{'story_id': 'CSV-27710', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
@@ -1200,12 +1280,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>User navigates to the settings menu</t>
+          <t>Apply multiple filters and select the OR operator to add another filter.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Settings menu is displayed</t>
+          <t>Previously selected filters remain intact after the reload.</t>
         </is>
       </c>
       <c r="G22" s="2" t="n"/>
@@ -1219,25 +1299,37 @@
       <c r="K22" s="2" t="n"/>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Generated from Azure DevOps story: User Management: Ability for user to reset password</t>
+          <t>Ensures that existing filters are preserved during the reload.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n"/>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>UI_UX_CONSISTENCY - Smooth Reload Experience</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>smooth_reload_experience</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-27710', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+        </is>
+      </c>
       <c r="D23" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>User selects 'Reset Password' option</t>
+          <t>Apply a filter and select the OR operator to add another filter.</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Password reset form is displayed</t>
+          <t>The reload is smooth with no flicker or UI reset.</t>
         </is>
       </c>
       <c r="G23" s="3" t="n"/>
@@ -1249,23 +1341,39 @@
       <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n"/>
       <c r="K23" s="3" t="n"/>
-      <c r="L23" s="3" t="n"/>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>Checks for a seamless user experience during reload.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="2" t="n"/>
-      <c r="C24" s="2" t="n"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>ASYNC_TIMING - Filter Results Update Automatically</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>filter_results_update_automatically</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-27710', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+        </is>
+      </c>
       <c r="D24" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>User enters their current password and a new valid password, then submits the form</t>
+          <t>Apply a filter, select the OR operator, and add another filter.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>New password is accepted and a success message is displayed</t>
+          <t>Results update automatically without requiring manual refresh.</t>
         </is>
       </c>
       <c r="G24" s="2" t="n"/>
@@ -1277,22 +1385,26 @@
       <c r="I24" s="2" t="n"/>
       <c r="J24" s="2" t="n"/>
       <c r="K24" s="2" t="n"/>
-      <c r="L24" s="2" t="n"/>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Ensures that results are updated in real-time as filters are applied.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Edge Case: Password Reset with Weak Password</t>
+          <t>ERROR_FAILURE - Handle Filter Reload Failure Gracefully</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>edge_case_weak_password</t>
+          <t>handle_filter_reload_failure_gracefully</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-3', 'story_title': 'User Management: Ability for user to reset password'}</t>
+          <t>{'story_id': 'CSV-27710', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1300,12 +1412,12 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>User accesses the password reset option in the settings menu</t>
+          <t>Simulate a network failure during filter reload.</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Password reset form is shown</t>
+          <t>A nonintrusive error message is displayed and user's filter selections are preserved.</t>
         </is>
       </c>
       <c r="G25" s="3" t="n"/>
@@ -1319,25 +1431,37 @@
       <c r="K25" s="3" t="n"/>
       <c r="L25" s="3" t="inlineStr">
         <is>
-          <t>Generated from Azure DevOps story: User Management: Ability for user to reset password</t>
+          <t>Tests error handling and user notification during reload failures.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>REMOVAL_DESELECTION - Undo OR Operator Selection</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>undo_or_operator_selection</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-27710', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+        </is>
+      </c>
       <c r="D26" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>User inputs their current password and a new weak password, then submits the form</t>
+          <t>Apply a filter, select the OR operator, then deselect it.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Form highlights the new password as too weak and prompts for a stronger password</t>
+          <t>The OR operator is removed and the filter panel returns to its previous state.</t>
         </is>
       </c>
       <c r="G26" s="2" t="n"/>
@@ -1349,22 +1473,26 @@
       <c r="I26" s="2" t="n"/>
       <c r="J26" s="2" t="n"/>
       <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="n"/>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Verifies that users can undo their selection of the OR operator.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Error Scenario: Incorrect Current Password</t>
+          <t>BOUNDARY_EMPTY - No Filters Applied</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>error_scenario_incorrect_current_password</t>
+          <t>no_filters_applied</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-3', 'story_title': 'User Management: Ability for user to reset password'}</t>
+          <t>{'story_id': 'CSV-27710', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1372,12 +1500,12 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>User navigates to the password reset option in the settings menu</t>
+          <t>Open the Advanced Filter section without applying any filters.</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Password reset form is displayed</t>
+          <t>Filter panel displays all available filter options.</t>
         </is>
       </c>
       <c r="G27" s="3" t="n"/>
@@ -1391,25 +1519,37 @@
       <c r="K27" s="3" t="n"/>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>Generated from Azure DevOps story: User Management: Ability for user to reset password</t>
+          <t>Checks system behavior when no filters are applied.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n"/>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>MIXED_DATA - Filters with Mixed Metadata</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>filters_with_mixed_metadata</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-27710', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+        </is>
+      </c>
       <c r="D28" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>User enters an incorrect current password and a new valid password, then submits the form</t>
+          <t>Apply filters that include assets with mixed metadata and select the OR operator.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>An error is displayed indicating the current password is incorrect</t>
+          <t>Filter panel updates to show options relevant to the mixed metadata.</t>
         </is>
       </c>
       <c r="G28" s="2" t="n"/>
@@ -1421,7 +1561,11 @@
       <c r="I28" s="2" t="n"/>
       <c r="J28" s="2" t="n"/>
       <c r="K28" s="2" t="n"/>
-      <c r="L28" s="2" t="n"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Ensures that the system can handle and display mixed metadata correctly.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Added Frontend for the QA Test Agent, improved report statistics
</commit_message>
<xml_diff>
--- a/outputs/qa_testing_agent/test_inputs/devops_tests.xlsx
+++ b/outputs/qa_testing_agent/test_inputs/devops_tests.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -526,17 +526,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>HAPPY_PATH - Auto-populate additional tags after results load</t>
+          <t>HAPPY_PATH - Category/Field Name filter visibility</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>auto_populate_tags_after_results_load</t>
+          <t>category_field_filter_visible_after_search</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-60210', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
@@ -544,12 +544,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>User selects Tag A from the filter panel.</t>
+          <t>Perform a keyword search using the DAM search bar.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Assets associated with Tag A are displayed.</t>
+          <t>The 'Category / Field Name' filter block appears below the 'Advanced Filters' section and is visible by default.</t>
         </is>
       </c>
       <c r="G2" s="2" t="n"/>
@@ -563,25 +563,37 @@
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Ensures basic functionality of auto-populating additional tags.</t>
+          <t>Ensures the filter block is always visible after a search.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n"/>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>MULTI_COMBINATION - Selecting multiple metadata fields</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>select_multiple_metadata_fields</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+        </is>
+      </c>
       <c r="D3" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Wait for the results to finish loading.</t>
+          <t>Perform a keyword search for 'Apple'.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Additional tags associated with the returned assets appear in the filter panel.</t>
+          <t>Search results are displayed with the 'Category / Field Name' filter block visible.</t>
         </is>
       </c>
       <c r="G3" s="3" t="n"/>
@@ -593,35 +605,27 @@
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Tests the AND logic when multiple fields are selected.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>MULTI_COMBINATION - Select multiple tags for filtering</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>select_multiple_tags_for_filtering</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-60210', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
       <c r="D4" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>User selects Tag A and Tag B from the filter panel.</t>
+          <t>Select 'Title' and 'Tags' from the 'Category / Field Name' filter block.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Assets associated with both Tag A and Tag B are displayed.</t>
+          <t>Results update to show only assets where 'Apple' appears in both 'Title' and 'Tags'.</t>
         </is>
       </c>
       <c r="G4" s="2" t="n"/>
@@ -633,27 +637,35 @@
       <c r="I4" s="2" t="n"/>
       <c r="J4" s="2" t="n"/>
       <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>Tests the system's ability to handle multiple tag selections.</t>
-        </is>
-      </c>
+      <c r="L4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>SEQUENTIAL_REFINEMENT - Drill down using multiple filters</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>drill_down_with_multiple_filters</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+        </is>
+      </c>
       <c r="D5" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Wait for the results to finish loading.</t>
+          <t>Perform a keyword search for 'Vietnamese'.</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Additional tags associated with the returned assets appear in the filter panel.</t>
+          <t>Search results are displayed with the 'Category / Field Name' filter block visible.</t>
         </is>
       </c>
       <c r="G5" s="3" t="n"/>
@@ -665,35 +677,27 @@
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
       <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n"/>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Ensures sequential refinement of search results using multiple filters.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>SEQUENTIAL_REFINEMENT - Further refine results with additional tags</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>further_refine_with_additional_tags</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-60210', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
       <c r="D6" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>User selects Tag A from the filter panel.</t>
+          <t>Select 'Language' from the 'Category / Field Name' filter block.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Assets associated with Tag A are displayed.</t>
+          <t>Results update to show only assets where 'Vietnamese' appears in the 'Language' field.</t>
         </is>
       </c>
       <c r="G6" s="2" t="n"/>
@@ -705,27 +709,23 @@
       <c r="I6" s="2" t="n"/>
       <c r="J6" s="2" t="n"/>
       <c r="K6" s="2" t="n"/>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>Verifies that users can refine results using newly populated tags.</t>
-        </is>
-      </c>
+      <c r="L6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
       <c r="B7" s="3" t="n"/>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Wait for the results to finish loading.</t>
+          <t>Select 'Description' from the 'Category / Field Name' filter block.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Additional tags associated with the returned assets appear in the filter panel.</t>
+          <t>Results update to show only assets where 'Vietnamese' appears in both 'Language' and 'Description' fields.</t>
         </is>
       </c>
       <c r="G7" s="3" t="n"/>
@@ -740,20 +740,32 @@
       <c r="L7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>STATE_PERSISTENCE - Saved search retains filter selections</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>saved_search_retains_filters</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+        </is>
+      </c>
       <c r="D8" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>User selects an additional tag from the newly populated tags.</t>
+          <t>Perform a keyword search for 'Apple' and select 'Title' and 'Tags' in the 'Category / Field Name' filter block.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Assets are further filtered based on the additional tag.</t>
+          <t>Results update to show assets where 'Apple' appears in 'Title' and 'Tags'.</t>
         </is>
       </c>
       <c r="G8" s="2" t="n"/>
@@ -765,35 +777,27 @@
       <c r="I8" s="2" t="n"/>
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="n"/>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Verifies that saved searches retain all filter selections.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>STATE_PERSISTENCE - User-selected tags remain highlighted</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>user_selected_tags_remain_highlighted</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-60210', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
-        </is>
-      </c>
+      <c r="A9" s="3" t="n"/>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
       <c r="D9" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>User selects Tag A from the filter panel.</t>
+          <t>Click 'Save Search'.</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Tag A is highlighted in the filter panel.</t>
+          <t>Search is saved with current filters.</t>
         </is>
       </c>
       <c r="G9" s="3" t="n"/>
@@ -805,27 +809,23 @@
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
       <c r="K9" s="3" t="n"/>
-      <c r="L9" s="3" t="inlineStr">
-        <is>
-          <t>Ensures user selections persist after results load.</t>
-        </is>
-      </c>
+      <c r="L9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
       <c r="B10" s="2" t="n"/>
       <c r="C10" s="2" t="n"/>
       <c r="D10" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Wait for the results to finish loading.</t>
+          <t>Re-open the saved search.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Tag A remains highlighted, and additional tags appear.</t>
+          <t>The keyword, 'Advanced Filters', and 'Category / Field Name' selections are restored.</t>
         </is>
       </c>
       <c r="G10" s="2" t="n"/>
@@ -842,17 +842,17 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>BUSINESS_RULES - Display all tags associated with returned results</t>
+          <t>UI_UX_CONSISTENCY - Visual consistency of filter block</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>display_all_tags_associated_with_results</t>
+          <t>filter_block_visual_consistency</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-60210', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
@@ -860,12 +860,12 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>User selects Tag A from the filter panel.</t>
+          <t>Perform a keyword search using the DAM search bar.</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Assets associated with Tag A are displayed.</t>
+          <t>The 'Category / Field Name' filter block visually matches the design of the 'Advanced Filters' area.</t>
         </is>
       </c>
       <c r="G11" s="3" t="n"/>
@@ -879,25 +879,37 @@
       <c r="K11" s="3" t="n"/>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>Validates that no tags are omitted from the filter panel.</t>
+          <t>Ensures visual consistency with existing UI elements.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>REMOVAL_DESELECTION - Deselecting a metadata field</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>deselect_metadata_field</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+        </is>
+      </c>
       <c r="D12" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Wait for the results to finish loading.</t>
+          <t>Perform a keyword search for 'Apple' and select 'Title' in the 'Category / Field Name' filter block.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>All tags associated with the returned assets are displayed in the filter panel.</t>
+          <t>Results update to show assets where 'Apple' appears in 'Title'.</t>
         </is>
       </c>
       <c r="G12" s="2" t="n"/>
@@ -909,35 +921,27 @@
       <c r="I12" s="2" t="n"/>
       <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="n"/>
-      <c r="L12" s="2" t="n"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Tests the removal of a filter and its effect on search results.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>UI_UX_CONSISTENCY - Consistent styling of newly added tags</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>consistent_styling_of_newly_added_tags</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-60210', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
-        </is>
-      </c>
+      <c r="A13" s="3" t="n"/>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="3" t="n"/>
       <c r="D13" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>User selects Tag A from the filter panel.</t>
+          <t>Deselect 'Title' by removing the chip/tag.</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Assets associated with Tag A are displayed.</t>
+          <t>Results update to include all assets with 'Apple' in any metadata field.</t>
         </is>
       </c>
       <c r="G13" s="3" t="n"/>
@@ -949,27 +953,35 @@
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
       <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="inlineStr">
-        <is>
-          <t>Checks for visual consistency in the filter panel.</t>
-        </is>
-      </c>
+      <c r="L13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>CLEAR_RESET_ALL - Clearing all search parameters</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>clear_all_search_parameters</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+        </is>
+      </c>
       <c r="D14" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Wait for the results to finish loading.</t>
+          <t>Perform a keyword search for 'Apple' and select 'Title' and 'Tags' in the 'Category / Field Name' filter block.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Newly added tags appear with the same style as existing tags.</t>
+          <t>Results update to show assets where 'Apple' appears in 'Title' and 'Tags'.</t>
         </is>
       </c>
       <c r="G14" s="2" t="n"/>
@@ -981,35 +993,27 @@
       <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="n"/>
       <c r="K14" s="2" t="n"/>
-      <c r="L14" s="2" t="n"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Ensures the 'Clear Search' functionality resets all filters and search parameters.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>BOUNDARY_EMPTY - Handle zero results gracefully</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>handle_zero_results_gracefully</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-60210', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
-        </is>
-      </c>
+      <c r="A15" s="3" t="n"/>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
       <c r="D15" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>User selects a tag with no associated assets.</t>
+          <t>Click 'Clear Search'.</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>No assets are displayed, and the filter panel shows no additional tags.</t>
+          <t>The keyword, all 'Advanced Filters', and 'Category / Field Name' selections are removed.</t>
         </is>
       </c>
       <c r="G15" s="3" t="n"/>
@@ -1021,26 +1025,22 @@
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
       <c r="K15" s="3" t="n"/>
-      <c r="L15" s="3" t="inlineStr">
-        <is>
-          <t>Tests system behavior when no results are returned.</t>
-        </is>
-      </c>
+      <c r="L15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>ASYNC_TIMING - Seamless UI update after loading</t>
+          <t>BOUNDARY_EMPTY - No results for a selected field</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>seamless_ui_update_after_loading</t>
+          <t>no_results_for_selected_field</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-60210', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
@@ -1048,12 +1048,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>User selects Tag A from the filter panel.</t>
+          <t>Perform a keyword search for 'Apple'.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Assets associated with Tag A are displayed.</t>
+          <t>Search results are displayed with the 'Category / Field Name' filter block visible.</t>
         </is>
       </c>
       <c r="G16" s="2" t="n"/>
@@ -1067,7 +1067,7 @@
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Ensures smooth UI transitions during asynchronous operations.</t>
+          <t>Tests behavior when a selected field has no matching results.</t>
         </is>
       </c>
     </row>
@@ -1080,12 +1080,12 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Observe the UI during and after the loading process.</t>
+          <t>Select 'Language' from the 'Category / Field Name' filter block.</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>The UI updates seamlessly without flickering or delay.</t>
+          <t>No results are displayed as 'Apple' does not appear in the 'Language' field.</t>
         </is>
       </c>
       <c r="G17" s="3" t="n"/>
@@ -1102,17 +1102,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>ERROR_FAILURE - Network error during tag population</t>
+          <t>MIXED_DATA - Mixed metadata fields with varying counts</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>network_error_during_tag_population</t>
+          <t>mixed_metadata_fields_varying_counts</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-60210', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
@@ -1120,12 +1120,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network error after selecting Tag A.</t>
+          <t>Perform a keyword search for 'Apple'.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>An error message is displayed, and the filter panel does not update with additional tags.</t>
+          <t>The filter block shows fields with counts: Title (3), Description (6), Tags (10), Language (0), Custom Field: Category (4).</t>
         </is>
       </c>
       <c r="G18" s="2" t="n"/>
@@ -1139,37 +1139,25 @@
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Tests system resilience to network failures during tag population.</t>
+          <t>Ensures correct count display and filtering with mixed data.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>HAPPY_PATH - Full Filter Reload on OR Operator Selection</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>full_filter_reload_on_or_operator_selection</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-27710', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
-        </is>
-      </c>
+      <c r="A19" s="3" t="n"/>
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="3" t="n"/>
       <c r="D19" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Navigate to the Advanced Filter section and apply an initial filter.</t>
+          <t>Select 'Description' and 'Custom Field: Category'.</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Initial filter is applied and visible in the filter panel.</t>
+          <t>Results update to show assets where 'Apple' appears in both 'Description' and 'Custom Field: Category'.</t>
         </is>
       </c>
       <c r="G19" s="3" t="n"/>
@@ -1181,27 +1169,35 @@
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
       <c r="K19" s="3" t="n"/>
-      <c r="L19" s="3" t="inlineStr">
-        <is>
-          <t>Ensures the core functionality of filter panel reloading is working as expected.</t>
-        </is>
-      </c>
+      <c r="L19" s="3" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n"/>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="n"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>PERFORMANCE_SCALE - Large dataset response time</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>large_dataset_response_time</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+        </is>
+      </c>
       <c r="D20" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Select the OR operator to add an additional filter condition.</t>
+          <t>Perform a keyword search for a common term expected to return thousands of results.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>The entire filter panel reloads automatically.</t>
+          <t>The 'Category / Field Name' filter block and search results load within acceptable response time.</t>
         </is>
       </c>
       <c r="G20" s="2" t="n"/>
@@ -1213,22 +1209,26 @@
       <c r="I20" s="2" t="n"/>
       <c r="J20" s="2" t="n"/>
       <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="n"/>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Tests system performance with large datasets.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>BUSINESS_RULES - Updated Filter Options Based on Previous Selections</t>
+          <t>HAPPY_PATH - Auto-populate additional tags after results load</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>updated_filter_options_based_on_previous_selections</t>
+          <t>auto_populate_tags_after_results_load</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-27710', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+          <t>{'story_id': 'CSV-21294', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -1236,12 +1236,12 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Apply a filter and then select the OR operator to add another filter.</t>
+          <t>Select Tag A in the filter panel.</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Filter panel displays updated and relevant filter options based on previously applied filters.</t>
+          <t>Assets with Tag A are displayed.</t>
         </is>
       </c>
       <c r="G21" s="3" t="n"/>
@@ -1255,37 +1255,25 @@
       <c r="K21" s="3" t="n"/>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>Verifies that new filter options are relevant to the current context.</t>
+          <t>Ensures that additional tags are auto-populated after initial filter selection.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>STATE_PERSISTENCE - No Loss of Existing Filters After Reload</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>no_loss_of_existing_filters_after_reload</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-27710', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
-        </is>
-      </c>
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
       <c r="D22" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Apply multiple filters and select the OR operator to add another filter.</t>
+          <t>Wait for the results to finish loading.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Previously selected filters remain intact after the reload.</t>
+          <t>All tags associated with the returned assets, including Tag B, appear in the filter panel.</t>
         </is>
       </c>
       <c r="G22" s="2" t="n"/>
@@ -1297,26 +1285,22 @@
       <c r="I22" s="2" t="n"/>
       <c r="J22" s="2" t="n"/>
       <c r="K22" s="2" t="n"/>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>Ensures that existing filters are preserved during the reload.</t>
-        </is>
-      </c>
+      <c r="L22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>UI_UX_CONSISTENCY - Smooth Reload Experience</t>
+          <t>MULTI_COMBINATION - Multiple tags appear in filter panel</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>smooth_reload_experience</t>
+          <t>multiple_tags_appear_in_filter_panel</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-27710', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+          <t>{'story_id': 'CSV-21294', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -1324,12 +1308,12 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Apply a filter and select the OR operator to add another filter.</t>
+          <t>Select Tag X in the filter panel.</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>The reload is smooth with no flicker or UI reset.</t>
+          <t>Assets with Tag X are displayed.</t>
         </is>
       </c>
       <c r="G23" s="3" t="n"/>
@@ -1343,37 +1327,25 @@
       <c r="K23" s="3" t="n"/>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>Checks for a seamless user experience during reload.</t>
+          <t>Verifies that multiple related tags are populated in the filter panel.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>ASYNC_TIMING - Filter Results Update Automatically</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>filter_results_update_automatically</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-27710', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
-        </is>
-      </c>
+      <c r="A24" s="2" t="n"/>
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="2" t="n"/>
       <c r="D24" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Apply a filter, select the OR operator, and add another filter.</t>
+          <t>Wait for the results to finish loading.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Results update automatically without requiring manual refresh.</t>
+          <t>Tags Y and Z, associated with the returned assets, appear in the filter panel.</t>
         </is>
       </c>
       <c r="G24" s="2" t="n"/>
@@ -1385,26 +1357,22 @@
       <c r="I24" s="2" t="n"/>
       <c r="J24" s="2" t="n"/>
       <c r="K24" s="2" t="n"/>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>Ensures that results are updated in real-time as filters are applied.</t>
-        </is>
-      </c>
+      <c r="L24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>ERROR_FAILURE - Handle Filter Reload Failure Gracefully</t>
+          <t>SEQUENTIAL_REFINEMENT - Further filter using newly surfaced tags</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>handle_filter_reload_failure_gracefully</t>
+          <t>further_filter_with_new_tags</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-27710', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+          <t>{'story_id': 'CSV-21294', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1412,12 +1380,12 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Simulate a network failure during filter reload.</t>
+          <t>Select Tag A in the filter panel.</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>A nonintrusive error message is displayed and user's filter selections are preserved.</t>
+          <t>Assets with Tag A are displayed.</t>
         </is>
       </c>
       <c r="G25" s="3" t="n"/>
@@ -1431,37 +1399,25 @@
       <c r="K25" s="3" t="n"/>
       <c r="L25" s="3" t="inlineStr">
         <is>
-          <t>Tests error handling and user notification during reload failures.</t>
+          <t>Tests the ability to refine results using newly populated tags.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>REMOVAL_DESELECTION - Undo OR Operator Selection</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>undo_or_operator_selection</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-27710', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
-        </is>
-      </c>
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
       <c r="D26" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Apply a filter, select the OR operator, then deselect it.</t>
+          <t>Wait for the results to finish loading.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>The OR operator is removed and the filter panel returns to its previous state.</t>
+          <t>Additional tags appear in the filter panel.</t>
         </is>
       </c>
       <c r="G26" s="2" t="n"/>
@@ -1473,39 +1429,23 @@
       <c r="I26" s="2" t="n"/>
       <c r="J26" s="2" t="n"/>
       <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>Verifies that users can undo their selection of the OR operator.</t>
-        </is>
-      </c>
+      <c r="L26" s="2" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>BOUNDARY_EMPTY - No Filters Applied</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>no_filters_applied</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-27710', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
-        </is>
-      </c>
+      <c r="A27" s="3" t="n"/>
+      <c r="B27" s="3" t="n"/>
+      <c r="C27" s="3" t="n"/>
       <c r="D27" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Open the Advanced Filter section without applying any filters.</t>
+          <t>Select one of the newly surfaced tags.</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Filter panel displays all available filter options.</t>
+          <t>Asset list is further narrowed down based on the additional tag.</t>
         </is>
       </c>
       <c r="G27" s="3" t="n"/>
@@ -1517,26 +1457,22 @@
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
       <c r="K27" s="3" t="n"/>
-      <c r="L27" s="3" t="inlineStr">
-        <is>
-          <t>Checks system behavior when no filters are applied.</t>
-        </is>
-      </c>
+      <c r="L27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>MIXED_DATA - Filters with Mixed Metadata</t>
+          <t>STATE_PERSISTENCE - User-selected tags remain highlighted</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>filters_with_mixed_metadata</t>
+          <t>user_selected_tags_remain_highlighted</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-27710', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+          <t>{'story_id': 'CSV-21294', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
@@ -1544,12 +1480,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Apply filters that include assets with mixed metadata and select the OR operator.</t>
+          <t>Select Tag A in the filter panel.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Filter panel updates to show options relevant to the mixed metadata.</t>
+          <t>Tag A is highlighted in the filter panel.</t>
         </is>
       </c>
       <c r="G28" s="2" t="n"/>
@@ -1563,7 +1499,1295 @@
       <c r="K28" s="2" t="n"/>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>Ensures that the system can handle and display mixed metadata correctly.</t>
+          <t>Ensures user selections persist after results load.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="3" t="n"/>
+      <c r="C29" s="3" t="n"/>
+      <c r="D29" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Wait for the results to finish loading.</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Tag A remains highlighted even after additional tags appear.</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="n"/>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="n"/>
+      <c r="J29" s="3" t="n"/>
+      <c r="K29" s="3" t="n"/>
+      <c r="L29" s="3" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>BOUNDARY_EMPTY - No additional tags to populate</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>no_additional_tags_to_populate</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-21294', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Select Tag A in the filter panel.</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Assets with Tag A are displayed.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="n"/>
+      <c r="J30" s="2" t="n"/>
+      <c r="K30" s="2" t="n"/>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Tests the system behavior when no additional tags are available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n"/>
+      <c r="B31" s="3" t="n"/>
+      <c r="C31" s="3" t="n"/>
+      <c r="D31" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Wait for the results to finish loading.</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>No new tags appear in the filter panel if no additional tags are associated with the results.</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="n"/>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="n"/>
+      <c r="J31" s="3" t="n"/>
+      <c r="K31" s="3" t="n"/>
+      <c r="L31" s="3" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>UI_UX_CONSISTENCY - Newly added tags appear in consistent style</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>new_tags_appear_consistent_style</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-21294', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Select Tag A in the filter panel.</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Assets with Tag A are displayed.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="n"/>
+      <c r="J32" s="2" t="n"/>
+      <c r="K32" s="2" t="n"/>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Ensures visual consistency in the filter panel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n"/>
+      <c r="B33" s="3" t="n"/>
+      <c r="C33" s="3" t="n"/>
+      <c r="D33" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Wait for the results to finish loading.</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Newly added tags appear in the same style as existing tags in the filter panel.</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="n"/>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="n"/>
+      <c r="J33" s="3" t="n"/>
+      <c r="K33" s="3" t="n"/>
+      <c r="L33" s="3" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>BUSINESS_RULES - All tags associated with results are displayed</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>all_associated_tags_displayed</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-21294', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Select Tag A in the filter panel.</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Assets with Tag A are displayed.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="n"/>
+      <c r="J34" s="2" t="n"/>
+      <c r="K34" s="2" t="n"/>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Verifies that no tags are omitted from the filter panel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n"/>
+      <c r="B35" s="3" t="n"/>
+      <c r="C35" s="3" t="n"/>
+      <c r="D35" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Wait for the results to finish loading.</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>All tags associated with the returned assets are displayed in the filter panel.</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="n"/>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="n"/>
+      <c r="J35" s="3" t="n"/>
+      <c r="K35" s="3" t="n"/>
+      <c r="L35" s="3" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>ASYNC_TIMING - UI updates seamlessly after loader completes</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>ui_updates_seamlessly_after_loader</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-21294', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Select Tag A in the filter panel.</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Assets with Tag A are displayed.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="n"/>
+      <c r="J36" s="2" t="n"/>
+      <c r="K36" s="2" t="n"/>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Tests the smoothness of UI updates post-loading.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n"/>
+      <c r="B37" s="3" t="n"/>
+      <c r="C37" s="3" t="n"/>
+      <c r="D37" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Observe the filter panel as the results load.</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Filter panel updates seamlessly with new tags once loading completes.</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="n"/>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="n"/>
+      <c r="J37" s="3" t="n"/>
+      <c r="K37" s="3" t="n"/>
+      <c r="L37" s="3" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>HAPPY_PATH - Full filter reload on OR operator selection</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>full_filter_reload_on_or_operator_selection</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-68069', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Navigate to the Advanced Filter section.</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Advanced Filter section is displayed.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="n"/>
+      <c r="J38" s="2" t="n"/>
+      <c r="K38" s="2" t="n"/>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Ensures the core functionality of triggering a reload when OR is selected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n"/>
+      <c r="B39" s="3" t="n"/>
+      <c r="C39" s="3" t="n"/>
+      <c r="D39" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Apply a filter condition.</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Filter condition is applied and results are filtered accordingly.</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="n"/>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="n"/>
+      <c r="J39" s="3" t="n"/>
+      <c r="K39" s="3" t="n"/>
+      <c r="L39" s="3" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n"/>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Select the OR operator to add a new filter condition.</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>The filter panel reloads automatically.</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="n"/>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="n"/>
+      <c r="J40" s="2" t="n"/>
+      <c r="K40" s="2" t="n"/>
+      <c r="L40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>MULTI_COMBINATION - Applying multiple filters with OR operator</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>multiple_filters_with_or_operator</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-68069', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Apply multiple filters using the OR operator in the Advanced Filter section.</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Multiple filters are applied, and the filter panel reloads with updated options.</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="n"/>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="n"/>
+      <c r="J41" s="3" t="n"/>
+      <c r="K41" s="3" t="n"/>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>Tests the system's ability to handle multiple filters and reload correctly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>STATE_PERSISTENCE - Retain existing filters after reload</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>retain_existing_filters_after_reload</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-68069', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Apply a filter condition.</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Filter condition is applied.</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="n"/>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="n"/>
+      <c r="J42" s="2" t="n"/>
+      <c r="K42" s="2" t="n"/>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>Ensures that existing filters are not lost during the reload process.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n"/>
+      <c r="B43" s="3" t="n"/>
+      <c r="C43" s="3" t="n"/>
+      <c r="D43" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Select the OR operator to add another filter condition.</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>The filter panel reloads, and the existing filter condition remains intact.</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="n"/>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="n"/>
+      <c r="J43" s="3" t="n"/>
+      <c r="K43" s="3" t="n"/>
+      <c r="L43" s="3" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>UI_UX_CONSISTENCY - Smooth reload without flicker</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>smooth_reload_without_flicker</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-68069', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Apply a filter and select the OR operator.</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>The filter panel reloads smoothly without flicker or reset.</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="n"/>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="n"/>
+      <c r="J44" s="2" t="n"/>
+      <c r="K44" s="2" t="n"/>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>Validates the user experience during the reload process.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>BUSINESS_RULES - Updated filter options based on previous selections</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>updated_filter_options_based_on_previous_selections</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-68069', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Apply a filter condition.</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Filter condition is applied.</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="n"/>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="n"/>
+      <c r="J45" s="3" t="n"/>
+      <c r="K45" s="3" t="n"/>
+      <c r="L45" s="3" t="inlineStr">
+        <is>
+          <t>Ensures that the filter options are dynamically updated based on prior selections.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n"/>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Select the OR operator to add another filter condition.</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>The filter panel reloads with updated and relevant filter options.</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="n"/>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="n"/>
+      <c r="J46" s="2" t="n"/>
+      <c r="K46" s="2" t="n"/>
+      <c r="L46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>LIFECYCLE_TRANSITION - Filter results update automatically</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>filter_results_update_automatically</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-68069', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Apply a filter condition and select the OR operator.</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>The filter panel reloads, and results update automatically without manual refresh.</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="n"/>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="n"/>
+      <c r="J47" s="3" t="n"/>
+      <c r="K47" s="3" t="n"/>
+      <c r="L47" s="3" t="inlineStr">
+        <is>
+          <t>Checks the automatic update of results after applying new filters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>ERROR_FAILURE - Handling reload failure</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>handling_reload_failure</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-68069', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Simulate a network failure during filter reload.</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>A nonintrusive error message is displayed, and existing filter selections are preserved.</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="n"/>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="n"/>
+      <c r="J48" s="2" t="n"/>
+      <c r="K48" s="2" t="n"/>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>Tests the system's error handling capabilities during reload failures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>BOUNDARY_EMPTY - Applying OR operator with no initial filters</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>or_operator_with_no_initial_filters</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-68069', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Navigate to the Advanced Filter section without applying any initial filters.</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Advanced Filter section is displayed with no filters applied.</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="n"/>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="n"/>
+      <c r="J49" s="3" t="n"/>
+      <c r="K49" s="3" t="n"/>
+      <c r="L49" s="3" t="inlineStr">
+        <is>
+          <t>Ensures functionality when no initial filters are applied.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n"/>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Select the OR operator to add a new filter condition.</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>The filter panel reloads with available filter options.</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="n"/>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="n"/>
+      <c r="J50" s="2" t="n"/>
+      <c r="K50" s="2" t="n"/>
+      <c r="L50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>HAPPY_PATH - Display of Category / Field Name filter</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>category_filter_visible_after_search</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-43732', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Perform a keyword search using the DAM search bar.</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>The 'Category / Field Name' filter block appears below the 'Advanced Filters' section.</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Ensures the filter block is visible by default after a search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>UI_UX_CONSISTENCY - Visual styling of filter block</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>category_filter_visual_styling</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-43732', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Perform a keyword search using the DAM search bar.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>The 'Category / Field Name' filter block matches the chip/tag style of other filters in the Advanced Filters area.</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Checks for visual consistency with existing UI components.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>MULTI_COMBINATION - Selecting multiple metadata fields</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>select_multiple_metadata_fields</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-43732', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Perform a keyword search using the DAM search bar.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>The 'Category / Field Name' filter block displays with all searchable metadata fields.</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Tests the AND logic when multiple fields are selected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="D54" t="n">
+        <v>2</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Select 'Title' and 'Tags' from the filter block.</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>The results update to show assets where the keyword appears in both 'Title' and 'Tags' fields.</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>BOUNDARY_EMPTY - No results in a specific field</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>no_results_in_language_field</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-43732', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Perform a keyword search for 'Apple'.</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>The 'Category / Field Name' filter block shows 'Language (0)'.</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Verifies behavior when a field has zero matching results.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="D56" t="n">
+        <v>2</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Select 'Language' from the filter block.</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>No results are displayed as no assets have 'Apple' in the 'Language' field.</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>REMOVAL_DESELECTION - Removing a selected filter</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>remove_selected_filter_chip</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-43732', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Perform a keyword search and select 'Title' from the filter block.</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Results update to show assets with the keyword in the 'Title' field.</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Tests the dynamic update of results upon filter removal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="D58" t="n">
+        <v>2</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Remove the 'Title' chip from the selected filters.</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Results update to include all assets matching the original keyword search without field restrictions.</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>STATE_PERSISTENCE - Saving and restoring searches</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>save_and_restore_search_with_filters</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-43732', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Perform a keyword search and select 'Title' and 'Tags' from the filter block.</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Results update to show assets with the keyword in both 'Title' and 'Tags'.</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Ensures saved searches retain all filter selections.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="D60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Click 'Save Search' and name the search.</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Search is saved with all selected filters.</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="D61" t="n">
+        <v>3</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Reopen the saved search.</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>The keyword, Advanced Filters, and 'Category / Field Name' selections are restored.</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>CLEAR_RESET_ALL - Clearing all search parameters</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>clear_search_resets_all_filters</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-43732', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Perform a keyword search and select multiple fields from the filter block.</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Results update based on selected fields.</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Validates the complete reset functionality of the search interface.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="D63" t="n">
+        <v>2</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Click 'Clear Search'.</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>The keyword, all Advanced Filters, and 'Category / Field Name' selections are removed.</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>PERFORMANCE_SCALE - Handling large data sets</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>performance_with_large_metadata_fields</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-43732', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Perform a keyword search expected to return a large number of results.</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>The 'Category / Field Name' filter block displays without performance degradation.</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Tests system performance with large datasets and multiple metadata fields.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>ASYNC_TIMING - Loader states and updates</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>loader_state_during_filter_selection</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-43732', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Perform a keyword search and select a field from the filter block.</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>A loader appears while the results update, and disappears once the update is complete.</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Ensures smooth UI transitions during asynchronous updates.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Changes to Preconditions and Report
</commit_message>
<xml_diff>
--- a/outputs/qa_testing_agent/test_inputs/devops_tests.xlsx
+++ b/outputs/qa_testing_agent/test_inputs/devops_tests.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -536,7 +536,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+          <t>{'story_id': 'CSV-51284', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
@@ -563,14 +563,14 @@
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Ensures the filter block is always visible after a search.</t>
+          <t>Ensures the filter block is displayed after a search.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>MULTI_COMBINATION - Selecting multiple metadata fields</t>
+          <t>MULTI_COMBINATION - Select multiple metadata fields</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -580,7 +580,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+          <t>{'story_id': 'CSV-51284', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
@@ -588,12 +588,12 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Perform a keyword search for 'Apple'.</t>
+          <t>Perform a keyword search using the DAM search bar.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Search results are displayed with the 'Category / Field Name' filter block visible.</t>
+          <t>Search results and 'Category / Field Name' filter block are displayed.</t>
         </is>
       </c>
       <c r="G3" s="3" t="n"/>
@@ -620,12 +620,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Select 'Title' and 'Tags' from the 'Category / Field Name' filter block.</t>
+          <t>Select 'Title' and 'Tags' fields from the filter block.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Results update to show only assets where 'Apple' appears in both 'Title' and 'Tags'.</t>
+          <t>Search results update to show only assets where the keyword appears in both 'Title' and 'Tags' fields.</t>
         </is>
       </c>
       <c r="G4" s="2" t="n"/>
@@ -647,12 +647,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>drill_down_with_multiple_filters</t>
+          <t>refine_search_with_multiple_filters</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+          <t>{'story_id': 'CSV-51284', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
@@ -660,12 +660,12 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Perform a keyword search for 'Vietnamese'.</t>
+          <t>Perform a keyword search using the DAM search bar.</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Search results are displayed with the 'Category / Field Name' filter block visible.</t>
+          <t>Search results and 'Category / Field Name' filter block are displayed.</t>
         </is>
       </c>
       <c r="G5" s="3" t="n"/>
@@ -679,7 +679,7 @@
       <c r="K5" s="3" t="n"/>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>Ensures sequential refinement of search results using multiple filters.</t>
+          <t>Tests sequential refinement of search results.</t>
         </is>
       </c>
     </row>
@@ -692,12 +692,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Select 'Language' from the 'Category / Field Name' filter block.</t>
+          <t>Select 'Description' field from the filter block.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Results update to show only assets where 'Vietnamese' appears in the 'Language' field.</t>
+          <t>Search results update to show only assets where the keyword appears in the 'Description' field.</t>
         </is>
       </c>
       <c r="G6" s="2" t="n"/>
@@ -720,12 +720,12 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Select 'Description' from the 'Category / Field Name' filter block.</t>
+          <t>Select 'Language' field from the filter block.</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Results update to show only assets where 'Vietnamese' appears in both 'Language' and 'Description' fields.</t>
+          <t>Search results update to show only assets where the keyword appears in both 'Description' and 'Language' fields.</t>
         </is>
       </c>
       <c r="G7" s="3" t="n"/>
@@ -742,17 +742,17 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>STATE_PERSISTENCE - Saved search retains filter selections</t>
+          <t>STATE_PERSISTENCE - Saved search restores filters</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>saved_search_retains_filters</t>
+          <t>saved_search_restores_filters</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+          <t>{'story_id': 'CSV-51284', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
@@ -760,12 +760,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Perform a keyword search for 'Apple' and select 'Title' and 'Tags' in the 'Category / Field Name' filter block.</t>
+          <t>Perform a keyword search and select 'Title' and 'Tags' fields.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Results update to show assets where 'Apple' appears in 'Title' and 'Tags'.</t>
+          <t>Search results update to show assets matching the selected fields.</t>
         </is>
       </c>
       <c r="G8" s="2" t="n"/>
@@ -779,7 +779,7 @@
       <c r="K8" s="2" t="n"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Verifies that saved searches retain all filter selections.</t>
+          <t>Ensures saved searches restore all filter states.</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Re-open the saved search.</t>
+          <t>Reopen the saved search.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -842,7 +842,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>UI_UX_CONSISTENCY - Visual consistency of filter block</t>
+          <t>UI_UX_CONSISTENCY - Filter block visual consistency</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+          <t>{'story_id': 'CSV-51284', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
@@ -879,14 +879,14 @@
       <c r="K11" s="3" t="n"/>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>Ensures visual consistency with existing UI elements.</t>
+          <t>Checks for visual consistency in UI design.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>REMOVAL_DESELECTION - Deselecting a metadata field</t>
+          <t>REMOVAL_DESELECTION - Deselect a metadata field</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -896,7 +896,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+          <t>{'story_id': 'CSV-51284', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
@@ -904,12 +904,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Perform a keyword search for 'Apple' and select 'Title' in the 'Category / Field Name' filter block.</t>
+          <t>Perform a keyword search and select 'Title' field.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Results update to show assets where 'Apple' appears in 'Title'.</t>
+          <t>Search results update to show assets where the keyword appears in the 'Title' field.</t>
         </is>
       </c>
       <c r="G12" s="2" t="n"/>
@@ -923,7 +923,7 @@
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Tests the removal of a filter and its effect on search results.</t>
+          <t>Tests the removal of a selected filter and its impact on results.</t>
         </is>
       </c>
     </row>
@@ -936,12 +936,12 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Deselect 'Title' by removing the chip/tag.</t>
+          <t>Remove the 'Title' chip from the filter bar.</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Results update to include all assets with 'Apple' in any metadata field.</t>
+          <t>Search results update to show all assets without the 'Title' filter applied.</t>
         </is>
       </c>
       <c r="G13" s="3" t="n"/>
@@ -958,17 +958,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>CLEAR_RESET_ALL - Clearing all search parameters</t>
+          <t>CLEAR_RESET_ALL - Clear all filters and search</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>clear_all_search_parameters</t>
+          <t>clear_all_filters_and_search</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+          <t>{'story_id': 'CSV-51284', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
@@ -976,12 +976,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Perform a keyword search for 'Apple' and select 'Title' and 'Tags' in the 'Category / Field Name' filter block.</t>
+          <t>Perform a keyword search and select multiple fields.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Results update to show assets where 'Apple' appears in 'Title' and 'Tags'.</t>
+          <t>Search results update to show assets matching the selected fields.</t>
         </is>
       </c>
       <c r="G14" s="2" t="n"/>
@@ -995,7 +995,7 @@
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Ensures the 'Clear Search' functionality resets all filters and search parameters.</t>
+          <t>Ensures the clear function resets all search parameters.</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>The keyword, all 'Advanced Filters', and 'Category / Field Name' selections are removed.</t>
+          <t>The keyword, all 'Advanced Filters', and 'Category / Field Name' selections are removed, and the system returns to baseline.</t>
         </is>
       </c>
       <c r="G15" s="3" t="n"/>
@@ -1030,17 +1030,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>BOUNDARY_EMPTY - No results for a selected field</t>
+          <t>BOUNDARY_EMPTY - No assets match the filter</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>no_results_for_selected_field</t>
+          <t>no_assets_match_filter</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+          <t>{'story_id': 'CSV-51284', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
@@ -1048,12 +1048,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Perform a keyword search for 'Apple'.</t>
+          <t>Perform a keyword search using a term not present in any metadata field.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Search results are displayed with the 'Category / Field Name' filter block visible.</t>
+          <t>The 'Category / Field Name' filter block displays fields with a count of zero.</t>
         </is>
       </c>
       <c r="G16" s="2" t="n"/>
@@ -1067,7 +1067,7 @@
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Tests behavior when a selected field has no matching results.</t>
+          <t>Tests system behavior when no assets match the selected filter.</t>
         </is>
       </c>
     </row>
@@ -1080,12 +1080,12 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Select 'Language' from the 'Category / Field Name' filter block.</t>
+          <t>Select any field with a count of zero.</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>No results are displayed as 'Apple' does not appear in the 'Language' field.</t>
+          <t>Search results show zero assets.</t>
         </is>
       </c>
       <c r="G17" s="3" t="n"/>
@@ -1102,17 +1102,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>MIXED_DATA - Mixed metadata fields with varying counts</t>
+          <t>ERROR_FAILURE - Handle network error gracefully</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>mixed_metadata_fields_varying_counts</t>
+          <t>handle_network_error_gracefully</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
+          <t>{'story_id': 'CSV-51284', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
@@ -1120,12 +1120,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Perform a keyword search for 'Apple'.</t>
+          <t>Simulate a network error during a keyword search.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>The filter block shows fields with counts: Title (3), Description (6), Tags (10), Language (0), Custom Field: Category (4).</t>
+          <t>An error message is displayed, and the 'Category / Field Name' filter block does not appear.</t>
         </is>
       </c>
       <c r="G18" s="2" t="n"/>
@@ -1139,25 +1139,37 @@
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Ensures correct count display and filtering with mixed data.</t>
+          <t>Ensures the system handles network errors without crashing.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n"/>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>HAPPY_PATH - Auto-populate additional tags after results load</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>auto_populate_tags_after_results_load</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-42376', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+        </is>
+      </c>
       <c r="D19" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Select 'Description' and 'Custom Field: Category'.</t>
+          <t>User selects Tag A from the filter panel.</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Results update to show assets where 'Apple' appears in both 'Description' and 'Custom Field: Category'.</t>
+          <t>Assets with Tag A are displayed.</t>
         </is>
       </c>
       <c r="G19" s="3" t="n"/>
@@ -1169,35 +1181,27 @@
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
       <c r="K19" s="3" t="n"/>
-      <c r="L19" s="3" t="n"/>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>Ensures that additional tags are auto-populated after initial filter.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>PERFORMANCE_SCALE - Large dataset response time</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>large_dataset_response_time</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-42701', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
-        </is>
-      </c>
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
       <c r="D20" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Perform a keyword search for a common term expected to return thousands of results.</t>
+          <t>Wait for the results to finish loading.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>The 'Category / Field Name' filter block and search results load within acceptable response time.</t>
+          <t>Additional tags associated with the returned assets appear in the filter panel.</t>
         </is>
       </c>
       <c r="G20" s="2" t="n"/>
@@ -1209,26 +1213,22 @@
       <c r="I20" s="2" t="n"/>
       <c r="J20" s="2" t="n"/>
       <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>Tests system performance with large datasets.</t>
-        </is>
-      </c>
+      <c r="L20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>HAPPY_PATH - Auto-populate additional tags after results load</t>
+          <t>MULTI_COMBINATION - Select multiple tags for filtering</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>auto_populate_tags_after_results_load</t>
+          <t>select_multiple_tags_for_filtering</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-21294', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+          <t>{'story_id': 'CSV-42376', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -1236,12 +1236,12 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Select Tag A in the filter panel.</t>
+          <t>User selects Tag A and Tag B from the filter panel.</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Assets with Tag A are displayed.</t>
+          <t>Assets with both Tag A and Tag B are displayed.</t>
         </is>
       </c>
       <c r="G21" s="3" t="n"/>
@@ -1255,7 +1255,7 @@
       <c r="K21" s="3" t="n"/>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>Ensures that additional tags are auto-populated after initial filter selection.</t>
+          <t>Tests the system's ability to handle multiple tag selections.</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>All tags associated with the returned assets, including Tag B, appear in the filter panel.</t>
+          <t>Additional tags associated with the returned assets appear in the filter panel.</t>
         </is>
       </c>
       <c r="G22" s="2" t="n"/>
@@ -1290,17 +1290,17 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>MULTI_COMBINATION - Multiple tags appear in filter panel</t>
+          <t>SEQUENTIAL_REFINEMENT - Further refine results using additional tags</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>multiple_tags_appear_in_filter_panel</t>
+          <t>refine_results_using_additional_tags</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-21294', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+          <t>{'story_id': 'CSV-42376', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -1308,12 +1308,12 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Select Tag X in the filter panel.</t>
+          <t>User selects Tag A from the filter panel.</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Assets with Tag X are displayed.</t>
+          <t>Assets with Tag A are displayed.</t>
         </is>
       </c>
       <c r="G23" s="3" t="n"/>
@@ -1327,7 +1327,7 @@
       <c r="K23" s="3" t="n"/>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>Verifies that multiple related tags are populated in the filter panel.</t>
+          <t>Validates the ability to drill down results using newly surfaced tags.</t>
         </is>
       </c>
     </row>
@@ -1345,7 +1345,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Tags Y and Z, associated with the returned assets, appear in the filter panel.</t>
+          <t>Additional tags appear in the filter panel.</t>
         </is>
       </c>
       <c r="G24" s="2" t="n"/>
@@ -1360,32 +1360,20 @@
       <c r="L24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>SEQUENTIAL_REFINEMENT - Further filter using newly surfaced tags</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>further_filter_with_new_tags</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-21294', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
-        </is>
-      </c>
+      <c r="A25" s="3" t="n"/>
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="3" t="n"/>
       <c r="D25" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Select Tag A in the filter panel.</t>
+          <t>User selects an additional tag from the newly populated options.</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Assets with Tag A are displayed.</t>
+          <t>Assets are further refined based on the additional tag.</t>
         </is>
       </c>
       <c r="G25" s="3" t="n"/>
@@ -1397,27 +1385,35 @@
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
       <c r="K25" s="3" t="n"/>
-      <c r="L25" s="3" t="inlineStr">
-        <is>
-          <t>Tests the ability to refine results using newly populated tags.</t>
-        </is>
-      </c>
+      <c r="L25" s="3" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>STATE_PERSISTENCE - Ensure selected tags remain highlighted</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>selected_tags_remain_highlighted</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-42376', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+        </is>
+      </c>
       <c r="D26" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Wait for the results to finish loading.</t>
+          <t>User selects Tag A from the filter panel.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Additional tags appear in the filter panel.</t>
+          <t>Tag A is highlighted in the filter panel.</t>
         </is>
       </c>
       <c r="G26" s="2" t="n"/>
@@ -1429,23 +1425,27 @@
       <c r="I26" s="2" t="n"/>
       <c r="J26" s="2" t="n"/>
       <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="n"/>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Checks that user-selected tags persist visually after loading.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n"/>
       <c r="B27" s="3" t="n"/>
       <c r="C27" s="3" t="n"/>
       <c r="D27" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Select one of the newly surfaced tags.</t>
+          <t>Wait for the results to finish loading.</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Asset list is further narrowed down based on the additional tag.</t>
+          <t>Tag A remains highlighted, and additional tags appear.</t>
         </is>
       </c>
       <c r="G27" s="3" t="n"/>
@@ -1462,17 +1462,17 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>STATE_PERSISTENCE - User-selected tags remain highlighted</t>
+          <t>BUSINESS_RULES - Display all tags associated with returned results</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>user_selected_tags_remain_highlighted</t>
+          <t>display_all_associated_tags</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-21294', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+          <t>{'story_id': 'CSV-42376', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
@@ -1480,12 +1480,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Select Tag A in the filter panel.</t>
+          <t>User selects Tag A from the filter panel.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Tag A is highlighted in the filter panel.</t>
+          <t>Assets with Tag A are displayed.</t>
         </is>
       </c>
       <c r="G28" s="2" t="n"/>
@@ -1499,7 +1499,7 @@
       <c r="K28" s="2" t="n"/>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>Ensures user selections persist after results load.</t>
+          <t>Ensures no tags are omitted from the filter panel.</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Tag A remains highlighted even after additional tags appear.</t>
+          <t>All tags associated with the returned assets are displayed in the filter panel.</t>
         </is>
       </c>
       <c r="G29" s="3" t="n"/>
@@ -1534,17 +1534,17 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>BOUNDARY_EMPTY - No additional tags to populate</t>
+          <t>UI_UX_CONSISTENCY - Consistent styling of newly added tags</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>no_additional_tags_to_populate</t>
+          <t>consistent_styling_of_new_tags</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-21294', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+          <t>{'story_id': 'CSV-42376', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Select Tag A in the filter panel.</t>
+          <t>User selects Tag A from the filter panel.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1571,7 +1571,7 @@
       <c r="K30" s="2" t="n"/>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Tests the system behavior when no additional tags are available.</t>
+          <t>Verifies visual consistency of the filter panel.</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>No new tags appear in the filter panel if no additional tags are associated with the results.</t>
+          <t>Newly added tags appear with the same styling as existing tags.</t>
         </is>
       </c>
       <c r="G31" s="3" t="n"/>
@@ -1606,17 +1606,17 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>UI_UX_CONSISTENCY - Newly added tags appear in consistent style</t>
+          <t>BOUNDARY_EMPTY - No additional tags available</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>new_tags_appear_consistent_style</t>
+          <t>no_additional_tags_available</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-21294', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+          <t>{'story_id': 'CSV-42376', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Select Tag A in the filter panel.</t>
+          <t>User selects Tag A from the filter panel.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1643,7 +1643,7 @@
       <c r="K32" s="2" t="n"/>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Ensures visual consistency in the filter panel.</t>
+          <t>Handles the case where no additional tags are available.</t>
         </is>
       </c>
     </row>
@@ -1661,7 +1661,7 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Newly added tags appear in the same style as existing tags in the filter panel.</t>
+          <t>No additional tags appear if none are associated with the returned assets.</t>
         </is>
       </c>
       <c r="G33" s="3" t="n"/>
@@ -1678,17 +1678,17 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>BUSINESS_RULES - All tags associated with results are displayed</t>
+          <t>ASYNC_TIMING - Loader states and UI update</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>all_associated_tags_displayed</t>
+          <t>loader_states_and_ui_update</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-21294', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+          <t>{'story_id': 'CSV-42376', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Select Tag A in the filter panel.</t>
+          <t>User selects Tag A from the filter panel.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -1715,7 +1715,7 @@
       <c r="K34" s="2" t="n"/>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>Verifies that no tags are omitted from the filter panel.</t>
+          <t>Ensures the UI updates seamlessly after loading.</t>
         </is>
       </c>
     </row>
@@ -1728,12 +1728,12 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Wait for the results to finish loading.</t>
+          <t>Observe the loader state until results finish loading.</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>All tags associated with the returned assets are displayed in the filter panel.</t>
+          <t>Loader disappears and additional tags appear in the filter panel.</t>
         </is>
       </c>
       <c r="G35" s="3" t="n"/>
@@ -1750,17 +1750,17 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>ASYNC_TIMING - UI updates seamlessly after loader completes</t>
+          <t>REMOVAL_DESELECTION - Deselect a tag and observe changes</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>ui_updates_seamlessly_after_loader</t>
+          <t>deselect_tag_and_observe_changes</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-21294', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
+          <t>{'story_id': 'CSV-42376', 'story_title': 'Auto-Populate Additional Tags in Filter After Results Load'}</t>
         </is>
       </c>
       <c r="D36" s="2" t="n">
@@ -1768,12 +1768,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Select Tag A in the filter panel.</t>
+          <t>User selects Tag A and Tag B from the filter panel.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Assets with Tag A are displayed.</t>
+          <t>Assets with both Tag A and Tag B are displayed.</t>
         </is>
       </c>
       <c r="G36" s="2" t="n"/>
@@ -1787,7 +1787,7 @@
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>Tests the smoothness of UI updates post-loading.</t>
+          <t>Tests the system's response to tag deselection.</t>
         </is>
       </c>
     </row>
@@ -1800,12 +1800,12 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Observe the filter panel as the results load.</t>
+          <t>User deselects Tag B.</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Filter panel updates seamlessly with new tags once loading completes.</t>
+          <t>Assets are updated to show only those with Tag A.</t>
         </is>
       </c>
       <c r="G37" s="3" t="n"/>
@@ -1822,17 +1822,17 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>HAPPY_PATH - Full filter reload on OR operator selection</t>
+          <t>HAPPY_PATH - Full Filter Reload on OR Operator Selection</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>full_filter_reload_on_or_operator_selection</t>
+          <t>full_filter_reload_on_or_operator</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-68069', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+          <t>{'story_id': 'CSV-52551', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
         </is>
       </c>
       <c r="D38" s="2" t="n">
@@ -1840,12 +1840,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Navigate to the Advanced Filter section.</t>
+          <t>Navigate to the Advanced Filter section and apply a filter.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Advanced Filter section is displayed.</t>
+          <t>Filter is applied and results are displayed.</t>
         </is>
       </c>
       <c r="G38" s="2" t="n"/>
@@ -1859,7 +1859,7 @@
       <c r="K38" s="2" t="n"/>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>Ensures the core functionality of triggering a reload when OR is selected.</t>
+          <t>Verifies that the filter panel reloads as expected when OR operator is selected.</t>
         </is>
       </c>
     </row>
@@ -1872,12 +1872,12 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Apply a filter condition.</t>
+          <t>Select the OR operator to add another filter condition.</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Filter condition is applied and results are filtered accordingly.</t>
+          <t>The entire filter panel reloads automatically.</t>
         </is>
       </c>
       <c r="G39" s="3" t="n"/>
@@ -1892,20 +1892,32 @@
       <c r="L39" s="3" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n"/>
-      <c r="B40" s="2" t="n"/>
-      <c r="C40" s="2" t="n"/>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>MULTI_COMBINATION - Updated Filter Options After Reload</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>updated_filter_options_after_reload</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-52551', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+        </is>
+      </c>
       <c r="D40" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Select the OR operator to add a new filter condition.</t>
+          <t>Apply multiple filters and select the OR operator.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>The filter panel reloads automatically.</t>
+          <t>Filter panel reloads with updated and relevant filter options.</t>
         </is>
       </c>
       <c r="G40" s="2" t="n"/>
@@ -1917,22 +1929,26 @@
       <c r="I40" s="2" t="n"/>
       <c r="J40" s="2" t="n"/>
       <c r="K40" s="2" t="n"/>
-      <c r="L40" s="2" t="n"/>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>Ensures that the filter options are updated based on previous selections and available metadata.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>MULTI_COMBINATION - Applying multiple filters with OR operator</t>
+          <t>STATE_PERSISTENCE - No Loss of Existing Filters</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>multiple_filters_with_or_operator</t>
+          <t>no_loss_of_existing_filters_after_reload</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-68069', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+          <t>{'story_id': 'CSV-52551', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
@@ -1940,12 +1956,12 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Apply multiple filters using the OR operator in the Advanced Filter section.</t>
+          <t>Apply a filter and select the OR operator to add another condition.</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>Multiple filters are applied, and the filter panel reloads with updated options.</t>
+          <t>Previously selected filters remain intact after the reload.</t>
         </is>
       </c>
       <c r="G41" s="3" t="n"/>
@@ -1959,24 +1975,24 @@
       <c r="K41" s="3" t="n"/>
       <c r="L41" s="3" t="inlineStr">
         <is>
-          <t>Tests the system's ability to handle multiple filters and reload correctly.</t>
+          <t>Checks that existing filters are preserved after applying the OR operator.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>STATE_PERSISTENCE - Retain existing filters after reload</t>
+          <t>UI_UX_CONSISTENCY - Smooth Reload Experience</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>retain_existing_filters_after_reload</t>
+          <t>smooth_reload_experience_no_flicker</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-68069', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+          <t>{'story_id': 'CSV-52551', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
         </is>
       </c>
       <c r="D42" s="2" t="n">
@@ -1984,12 +2000,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Apply a filter condition.</t>
+          <t>Apply a filter and select the OR operator.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Filter condition is applied.</t>
+          <t>The reload is smooth with no UI flicker or reset.</t>
         </is>
       </c>
       <c r="G42" s="2" t="n"/>
@@ -2003,25 +2019,37 @@
       <c r="K42" s="2" t="n"/>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>Ensures that existing filters are not lost during the reload process.</t>
+          <t>Verifies that the user experience is smooth during the reload process.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="n"/>
-      <c r="B43" s="3" t="n"/>
-      <c r="C43" s="3" t="n"/>
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>ASYNC_TIMING - Automatic Results Update</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>automatic_results_update_after_filter</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-52551', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+        </is>
+      </c>
       <c r="D43" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Select the OR operator to add another filter condition.</t>
+          <t>Apply a filter and select the OR operator.</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>The filter panel reloads, and the existing filter condition remains intact.</t>
+          <t>Results update automatically without requiring manual refresh.</t>
         </is>
       </c>
       <c r="G43" s="3" t="n"/>
@@ -2033,22 +2061,26 @@
       <c r="I43" s="3" t="n"/>
       <c r="J43" s="3" t="n"/>
       <c r="K43" s="3" t="n"/>
-      <c r="L43" s="3" t="n"/>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t>Ensures that results update automatically after the OR operator is applied.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>UI_UX_CONSISTENCY - Smooth reload without flicker</t>
+          <t>ERROR_FAILURE - Error Handling on Reload Failure</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>smooth_reload_without_flicker</t>
+          <t>error_handling_on_reload_failure</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-68069', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+          <t>{'story_id': 'CSV-52551', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
         </is>
       </c>
       <c r="D44" s="2" t="n">
@@ -2056,12 +2088,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Apply a filter and select the OR operator.</t>
+          <t>Simulate a network error during the filter reload process.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>The filter panel reloads smoothly without flicker or reset.</t>
+          <t>A nonintrusive error message is displayed and user’s filter selections are preserved.</t>
         </is>
       </c>
       <c r="G44" s="2" t="n"/>
@@ -2075,24 +2107,24 @@
       <c r="K44" s="2" t="n"/>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>Validates the user experience during the reload process.</t>
+          <t>Tests the system's ability to handle errors during the reload process.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>BUSINESS_RULES - Updated filter options based on previous selections</t>
+          <t>BOUNDARY_EMPTY - Single Filter Application</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>updated_filter_options_based_on_previous_selections</t>
+          <t>single_filter_application_with_or_operator</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-68069', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+          <t>{'story_id': 'CSV-52551', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
         </is>
       </c>
       <c r="D45" s="3" t="n">
@@ -2100,12 +2132,12 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Apply a filter condition.</t>
+          <t>Apply a single filter and select the OR operator.</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Filter condition is applied.</t>
+          <t>Filter panel reloads and displays relevant options for a single filter.</t>
         </is>
       </c>
       <c r="G45" s="3" t="n"/>
@@ -2119,25 +2151,37 @@
       <c r="K45" s="3" t="n"/>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t>Ensures that the filter options are dynamically updated based on prior selections.</t>
+          <t>Checks behavior when only one filter is applied with an OR operator.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n"/>
-      <c r="B46" s="2" t="n"/>
-      <c r="C46" s="2" t="n"/>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>REGRESSION - Unrelated Features Functionality</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>unrelated_features_still_function</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>{'story_id': 'CSV-52551', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+        </is>
+      </c>
       <c r="D46" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Select the OR operator to add another filter condition.</t>
+          <t>Perform unrelated actions such as sorting or pagination.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>The filter panel reloads with updated and relevant filter options.</t>
+          <t>Unrelated features function as expected after filter reload.</t>
         </is>
       </c>
       <c r="G46" s="2" t="n"/>
@@ -2149,22 +2193,26 @@
       <c r="I46" s="2" t="n"/>
       <c r="J46" s="2" t="n"/>
       <c r="K46" s="2" t="n"/>
-      <c r="L46" s="2" t="n"/>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>Ensures that unrelated features are not affected by the filter reload.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>LIFECYCLE_TRANSITION - Filter results update automatically</t>
+          <t>REMOVAL_DESELECTION - Undo OR Operator Selection</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>filter_results_update_automatically</t>
+          <t>undo_or_operator_selection</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-68069', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+          <t>{'story_id': 'CSV-52551', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
         </is>
       </c>
       <c r="D47" s="3" t="n">
@@ -2172,12 +2220,12 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Apply a filter condition and select the OR operator.</t>
+          <t>Apply a filter, select the OR operator, then deselect it.</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>The filter panel reloads, and results update automatically without manual refresh.</t>
+          <t>Filter panel reverts to the state before OR operator selection.</t>
         </is>
       </c>
       <c r="G47" s="3" t="n"/>
@@ -2191,24 +2239,24 @@
       <c r="K47" s="3" t="n"/>
       <c r="L47" s="3" t="inlineStr">
         <is>
-          <t>Checks the automatic update of results after applying new filters.</t>
+          <t>Tests the ability to undo the OR operator selection and revert to previous state.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>ERROR_FAILURE - Handling reload failure</t>
+          <t>PERFORMANCE_SCALE - Large Data Set Handling</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>handling_reload_failure</t>
+          <t>large_data_set_filter_reload_performance</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>{'story_id': 'CSV-68069', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
+          <t>{'story_id': 'CSV-52551', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
         </is>
       </c>
       <c r="D48" s="2" t="n">
@@ -2216,12 +2264,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Simulate a network failure during filter reload.</t>
+          <t>Apply filters on a large data set and select the OR operator.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>A nonintrusive error message is displayed, and existing filter selections are preserved.</t>
+          <t>Filter panel reloads efficiently without performance degradation.</t>
         </is>
       </c>
       <c r="G48" s="2" t="n"/>
@@ -2235,559 +2283,7 @@
       <c r="K48" s="2" t="n"/>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>Tests the system's error handling capabilities during reload failures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>BOUNDARY_EMPTY - Applying OR operator with no initial filters</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="inlineStr">
-        <is>
-          <t>or_operator_with_no_initial_filters</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-68069', 'story_title': 'Reload Filters When OR operator Is Selected in Advanced Filter'}</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>Navigate to the Advanced Filter section without applying any initial filters.</t>
-        </is>
-      </c>
-      <c r="F49" s="3" t="inlineStr">
-        <is>
-          <t>Advanced Filter section is displayed with no filters applied.</t>
-        </is>
-      </c>
-      <c r="G49" s="3" t="n"/>
-      <c r="H49" s="3" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="I49" s="3" t="n"/>
-      <c r="J49" s="3" t="n"/>
-      <c r="K49" s="3" t="n"/>
-      <c r="L49" s="3" t="inlineStr">
-        <is>
-          <t>Ensures functionality when no initial filters are applied.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="n"/>
-      <c r="B50" s="2" t="n"/>
-      <c r="C50" s="2" t="n"/>
-      <c r="D50" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>Select the OR operator to add a new filter condition.</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>The filter panel reloads with available filter options.</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="n"/>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="I50" s="2" t="n"/>
-      <c r="J50" s="2" t="n"/>
-      <c r="K50" s="2" t="n"/>
-      <c r="L50" s="2" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>HAPPY_PATH - Display of Category / Field Name filter</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>category_filter_visible_after_search</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-43732', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
-        </is>
-      </c>
-      <c r="D51" t="n">
-        <v>1</v>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Perform a keyword search using the DAM search bar.</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>The 'Category / Field Name' filter block appears below the 'Advanced Filters' section.</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>Ensures the filter block is visible by default after a search.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>UI_UX_CONSISTENCY - Visual styling of filter block</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>category_filter_visual_styling</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-43732', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
-        </is>
-      </c>
-      <c r="D52" t="n">
-        <v>1</v>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Perform a keyword search using the DAM search bar.</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>The 'Category / Field Name' filter block matches the chip/tag style of other filters in the Advanced Filters area.</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>Checks for visual consistency with existing UI components.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>MULTI_COMBINATION - Selecting multiple metadata fields</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>select_multiple_metadata_fields</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-43732', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
-        </is>
-      </c>
-      <c r="D53" t="n">
-        <v>1</v>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Perform a keyword search using the DAM search bar.</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>The 'Category / Field Name' filter block displays with all searchable metadata fields.</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>Tests the AND logic when multiple fields are selected.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="D54" t="n">
-        <v>2</v>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Select 'Title' and 'Tags' from the filter block.</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>The results update to show assets where the keyword appears in both 'Title' and 'Tags' fields.</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>BOUNDARY_EMPTY - No results in a specific field</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>no_results_in_language_field</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-43732', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
-        </is>
-      </c>
-      <c r="D55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Perform a keyword search for 'Apple'.</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>The 'Category / Field Name' filter block shows 'Language (0)'.</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>Verifies behavior when a field has zero matching results.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="D56" t="n">
-        <v>2</v>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Select 'Language' from the filter block.</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>No results are displayed as no assets have 'Apple' in the 'Language' field.</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>REMOVAL_DESELECTION - Removing a selected filter</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>remove_selected_filter_chip</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-43732', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
-        </is>
-      </c>
-      <c r="D57" t="n">
-        <v>1</v>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Perform a keyword search and select 'Title' from the filter block.</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>Results update to show assets with the keyword in the 'Title' field.</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>Tests the dynamic update of results upon filter removal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="D58" t="n">
-        <v>2</v>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Remove the 'Title' chip from the selected filters.</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>Results update to include all assets matching the original keyword search without field restrictions.</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>STATE_PERSISTENCE - Saving and restoring searches</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>save_and_restore_search_with_filters</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-43732', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
-        </is>
-      </c>
-      <c r="D59" t="n">
-        <v>1</v>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Perform a keyword search and select 'Title' and 'Tags' from the filter block.</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>Results update to show assets with the keyword in both 'Title' and 'Tags'.</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>Ensures saved searches retain all filter selections.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="D60" t="n">
-        <v>2</v>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Click 'Save Search' and name the search.</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>Search is saved with all selected filters.</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="D61" t="n">
-        <v>3</v>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Reopen the saved search.</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>The keyword, Advanced Filters, and 'Category / Field Name' selections are restored.</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>CLEAR_RESET_ALL - Clearing all search parameters</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>clear_search_resets_all_filters</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-43732', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
-        </is>
-      </c>
-      <c r="D62" t="n">
-        <v>1</v>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Perform a keyword search and select multiple fields from the filter block.</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>Results update based on selected fields.</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>Validates the complete reset functionality of the search interface.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="D63" t="n">
-        <v>2</v>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Click 'Clear Search'.</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>The keyword, all Advanced Filters, and 'Category / Field Name' selections are removed.</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>PERFORMANCE_SCALE - Handling large data sets</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>performance_with_large_metadata_fields</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-43732', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
-        </is>
-      </c>
-      <c r="D64" t="n">
-        <v>1</v>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Perform a keyword search expected to return a large number of results.</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>The 'Category / Field Name' filter block displays without performance degradation.</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>Tests system performance with large datasets and multiple metadata fields.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>ASYNC_TIMING - Loader states and updates</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>loader_state_during_filter_selection</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>{'story_id': 'CSV-43732', 'story_title': 'Add secondary “Category / Field Name” filter below Advanced Filters in DAM search results'}</t>
-        </is>
-      </c>
-      <c r="D65" t="n">
-        <v>1</v>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Perform a keyword search and select a field from the filter block.</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>A loader appears while the results update, and disappears once the update is complete.</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t>Ensures smooth UI transitions during asynchronous updates.</t>
+          <t>Evaluates system performance when handling large data sets during filter reload.</t>
         </is>
       </c>
     </row>

</xml_diff>